<commit_message>
prise en compte finale des commentaires
</commit_message>
<xml_diff>
--- a/date_periode_chasse.xlsx
+++ b/date_periode_chasse.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projets_Suzanne\Courlis\3) Data\1) data\Chasse\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projets_Suzanne\Courlis\Atlas_Courlis\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>2023/2024</t>
   </si>
@@ -65,6 +65,12 @@
   </si>
   <si>
     <t>Date de fermeture de la chasse</t>
+  </si>
+  <si>
+    <t>2017/2018</t>
+  </si>
+  <si>
+    <t>2016/2017</t>
   </si>
 </sst>
 </file>
@@ -443,7 +449,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="3" width="27.25" customWidth="1"/>
@@ -537,6 +543,28 @@
         <v>43496</v>
       </c>
     </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="1">
+        <v>42988</v>
+      </c>
+      <c r="C9" s="1">
+        <v>43131</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="1">
+        <v>42624</v>
+      </c>
+      <c r="C10" s="1">
+        <v>42766</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>